<commit_message>
make lookup table files, get rid of combustion delay in chamebr
</commit_message>
<xml_diff>
--- a/analysis/control_dev/First Princ + Data Driven/cstar_lookup_table.xlsx
+++ b/analysis/control_dev/First Princ + Data Driven/cstar_lookup_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Stuff\Capstone\capstone_throttleable_engine_2025-26\analysis\control_dev\First Princ + Data Driven\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6756E0C2-992C-46BA-B8CF-498373646876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E4A36C-A909-4108-982B-EECA1A5C4632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{0D6E4698-7F0B-418C-A5E1-474A908432D9}"/>
+    <workbookView xWindow="3204" yWindow="3204" windowWidth="17280" windowHeight="8880" xr2:uid="{0D6E4698-7F0B-418C-A5E1-474A908432D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,17 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>Pc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OF ratio </t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -405,575 +416,583 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B4B6FAD-C96D-4037-BEA6-8D82988DB960}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B1">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="C2">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C1">
+      <c r="D2">
         <v>1.133</v>
       </c>
-      <c r="D1">
+      <c r="E2">
         <v>1.167</v>
       </c>
-      <c r="E1">
+      <c r="F2">
         <v>1.2</v>
       </c>
-      <c r="F1">
+      <c r="G2">
         <v>1.2330000000000001</v>
       </c>
-      <c r="G1">
+      <c r="H2">
         <v>1.2669999999999999</v>
       </c>
-      <c r="H1">
+      <c r="I2">
         <v>1.3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3">
         <v>270</v>
       </c>
-      <c r="B2">
+      <c r="C3">
         <v>1152.2</v>
       </c>
-      <c r="C2">
+      <c r="D3">
         <v>1155.8</v>
       </c>
-      <c r="D2">
+      <c r="E3">
         <v>1158.5999999999999</v>
       </c>
-      <c r="E2">
+      <c r="F3">
         <v>1162</v>
       </c>
-      <c r="F2">
+      <c r="G3">
         <v>1167.5999999999999</v>
       </c>
-      <c r="G2">
+      <c r="H3">
         <v>1173.4000000000001</v>
       </c>
-      <c r="H2">
+      <c r="I3">
         <v>1179.0999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B4">
         <v>274</v>
       </c>
-      <c r="B3">
+      <c r="C4">
         <v>1152.4000000000001</v>
       </c>
-      <c r="C3">
+      <c r="D4">
         <v>1156.0999999999999</v>
       </c>
-      <c r="D3">
+      <c r="E4">
         <v>1158.8</v>
       </c>
-      <c r="E3">
+      <c r="F4">
         <v>1162.3</v>
       </c>
-      <c r="F3">
+      <c r="G4">
         <v>1167.9000000000001</v>
       </c>
-      <c r="G3">
+      <c r="H4">
         <v>1173.7</v>
       </c>
-      <c r="H3">
+      <c r="I4">
         <v>1179.3</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B5">
         <v>278</v>
       </c>
-      <c r="B4">
+      <c r="C5">
         <v>1152.7</v>
       </c>
-      <c r="C4">
+      <c r="D5">
         <v>1156.3</v>
       </c>
-      <c r="D4">
+      <c r="E5">
         <v>1159</v>
       </c>
-      <c r="E4">
+      <c r="F5">
         <v>1162.5</v>
       </c>
-      <c r="F4">
+      <c r="G5">
         <v>1168.0999999999999</v>
       </c>
-      <c r="G4">
+      <c r="H5">
         <v>1173.9000000000001</v>
       </c>
-      <c r="H4">
+      <c r="I5">
         <v>1179.5999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B6">
         <v>282</v>
       </c>
-      <c r="B5">
+      <c r="C6">
         <v>1152.9000000000001</v>
       </c>
-      <c r="C5">
+      <c r="D6">
         <v>1156.5</v>
       </c>
-      <c r="D5">
+      <c r="E6">
         <v>1159.2</v>
       </c>
-      <c r="E5">
+      <c r="F6">
         <v>1162.8</v>
       </c>
-      <c r="F5">
+      <c r="G6">
         <v>1168.4000000000001</v>
       </c>
-      <c r="G5">
+      <c r="H6">
         <v>1174.2</v>
       </c>
-      <c r="H5">
+      <c r="I6">
         <v>1179.9000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B7">
         <v>286</v>
       </c>
-      <c r="B6">
+      <c r="C7">
         <v>1153.0999999999999</v>
       </c>
-      <c r="C6">
+      <c r="D7">
         <v>1156.8</v>
       </c>
-      <c r="D6">
+      <c r="E7">
         <v>1159.5</v>
       </c>
-      <c r="E6">
+      <c r="F7">
         <v>1163.0999999999999</v>
       </c>
-      <c r="F6">
+      <c r="G7">
         <v>1168.7</v>
       </c>
-      <c r="G6">
+      <c r="H7">
         <v>1174.5</v>
       </c>
-      <c r="H6">
+      <c r="I7">
         <v>1180.2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B8">
         <v>290</v>
       </c>
-      <c r="B7">
+      <c r="C8">
         <v>1153.4000000000001</v>
       </c>
-      <c r="C7">
+      <c r="D8">
         <v>1157</v>
       </c>
-      <c r="D7">
+      <c r="E8">
         <v>1159.7</v>
       </c>
-      <c r="E7">
+      <c r="F8">
         <v>1163.3</v>
       </c>
-      <c r="F7">
+      <c r="G8">
         <v>1168.9000000000001</v>
       </c>
-      <c r="G7">
+      <c r="H8">
         <v>1174.7</v>
       </c>
-      <c r="H7">
+      <c r="I8">
         <v>1180.4000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B9">
         <v>294</v>
       </c>
-      <c r="B8">
+      <c r="C9">
         <v>1153.5999999999999</v>
       </c>
-      <c r="C8">
+      <c r="D9">
         <v>1157.2</v>
       </c>
-      <c r="D8">
+      <c r="E9">
         <v>1159.9000000000001</v>
       </c>
-      <c r="E8">
+      <c r="F9">
         <v>1163.5999999999999</v>
       </c>
-      <c r="F8">
+      <c r="G9">
         <v>1169.2</v>
       </c>
-      <c r="G8">
+      <c r="H9">
         <v>1175</v>
       </c>
-      <c r="H8">
+      <c r="I9">
         <v>1180.7</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B10">
         <v>298</v>
       </c>
-      <c r="B9">
+      <c r="C10">
         <v>1153.8</v>
       </c>
-      <c r="C9">
+      <c r="D10">
         <v>1157.4000000000001</v>
       </c>
-      <c r="D9">
+      <c r="E10">
         <v>1160.0999999999999</v>
       </c>
-      <c r="E9">
+      <c r="F10">
         <v>1163.9000000000001</v>
       </c>
-      <c r="F9">
+      <c r="G10">
         <v>1169.5</v>
       </c>
-      <c r="G9">
+      <c r="H10">
         <v>1175.3</v>
       </c>
-      <c r="H9">
+      <c r="I10">
         <v>1180.9000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B11">
         <v>302</v>
       </c>
-      <c r="B10">
+      <c r="C11">
         <v>1154</v>
       </c>
-      <c r="C10">
+      <c r="D11">
         <v>1157.5999999999999</v>
       </c>
-      <c r="D10">
+      <c r="E11">
         <v>1160.3</v>
       </c>
-      <c r="E10">
+      <c r="F11">
         <v>1164.0999999999999</v>
       </c>
-      <c r="F10">
+      <c r="G11">
         <v>1169.7</v>
       </c>
-      <c r="G10">
+      <c r="H11">
         <v>1175.5</v>
       </c>
-      <c r="H10">
+      <c r="I11">
         <v>1181.2</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B12">
         <v>306</v>
       </c>
-      <c r="B11">
+      <c r="C12">
         <v>1154.3</v>
       </c>
-      <c r="C11">
+      <c r="D12">
         <v>1157.8</v>
       </c>
-      <c r="D11">
+      <c r="E12">
         <v>1160.5</v>
       </c>
-      <c r="E11">
+      <c r="F12">
         <v>1164.4000000000001</v>
       </c>
-      <c r="F11">
+      <c r="G12">
         <v>1170</v>
       </c>
-      <c r="G11">
+      <c r="H12">
         <v>1175.8</v>
       </c>
-      <c r="H11">
+      <c r="I12">
         <v>1181.4000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B13">
         <v>310</v>
       </c>
-      <c r="B12">
+      <c r="C13">
         <v>1154.5</v>
       </c>
-      <c r="C12">
+      <c r="D13">
         <v>1158.0999999999999</v>
       </c>
-      <c r="D12">
+      <c r="E13">
         <v>1160.7</v>
       </c>
-      <c r="E12">
+      <c r="F13">
         <v>1164.5999999999999</v>
       </c>
-      <c r="F12">
+      <c r="G13">
         <v>1170.2</v>
       </c>
-      <c r="G12">
+      <c r="H13">
         <v>1176</v>
       </c>
-      <c r="H12">
+      <c r="I13">
         <v>1181.7</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B14">
         <v>314</v>
       </c>
-      <c r="B13">
+      <c r="C14">
         <v>1154.7</v>
       </c>
-      <c r="C13">
+      <c r="D14">
         <v>1158.3</v>
       </c>
-      <c r="D13">
+      <c r="E14">
         <v>1160.9000000000001</v>
       </c>
-      <c r="E13">
+      <c r="F14">
         <v>1164.9000000000001</v>
       </c>
-      <c r="F13">
+      <c r="G14">
         <v>1170.5</v>
       </c>
-      <c r="G13">
+      <c r="H14">
         <v>1176.3</v>
       </c>
-      <c r="H13">
+      <c r="I14">
         <v>1181.9000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B15">
         <v>318</v>
       </c>
-      <c r="B14">
+      <c r="C15">
         <v>1154.9000000000001</v>
       </c>
-      <c r="C14">
+      <c r="D15">
         <v>1158.5</v>
       </c>
-      <c r="D14">
+      <c r="E15">
         <v>1161.0999999999999</v>
       </c>
-      <c r="E14">
+      <c r="F15">
         <v>1165.0999999999999</v>
       </c>
-      <c r="F14">
+      <c r="G15">
         <v>1170.7</v>
       </c>
-      <c r="G14">
+      <c r="H15">
         <v>1176.5</v>
       </c>
-      <c r="H14">
+      <c r="I15">
         <v>1182.2</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B16">
         <v>322</v>
       </c>
-      <c r="B15">
+      <c r="C16">
         <v>1155.0999999999999</v>
       </c>
-      <c r="C15">
+      <c r="D16">
         <v>1158.7</v>
       </c>
-      <c r="D15">
+      <c r="E16">
         <v>1161.3</v>
       </c>
-      <c r="E15">
+      <c r="F16">
         <v>1165.3</v>
       </c>
-      <c r="F15">
+      <c r="G16">
         <v>1170.9000000000001</v>
       </c>
-      <c r="G15">
+      <c r="H16">
         <v>1176.7</v>
       </c>
-      <c r="H15">
+      <c r="I16">
         <v>1182.4000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B17">
         <v>326</v>
       </c>
-      <c r="B16">
+      <c r="C17">
         <v>1155.3</v>
       </c>
-      <c r="C16">
+      <c r="D17">
         <v>1158.9000000000001</v>
       </c>
-      <c r="D16">
+      <c r="E17">
         <v>1161.5</v>
       </c>
-      <c r="E16">
+      <c r="F17">
         <v>1165.5999999999999</v>
       </c>
-      <c r="F16">
+      <c r="G17">
         <v>1171.2</v>
       </c>
-      <c r="G16">
+      <c r="H17">
         <v>1177</v>
       </c>
-      <c r="H16">
+      <c r="I17">
         <v>1182.5999999999999</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B18">
         <v>330</v>
       </c>
-      <c r="B17">
+      <c r="C18">
         <v>1155.5</v>
       </c>
-      <c r="C17">
+      <c r="D18">
         <v>1159.0999999999999</v>
       </c>
-      <c r="D17">
+      <c r="E18">
         <v>1161.7</v>
       </c>
-      <c r="E17">
+      <c r="F18">
         <v>1165.8</v>
       </c>
-      <c r="F17">
+      <c r="G18">
         <v>1171.4000000000001</v>
       </c>
-      <c r="G17">
+      <c r="H18">
         <v>1177.2</v>
       </c>
-      <c r="H17">
+      <c r="I18">
         <v>1182.9000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B19">
         <v>334</v>
       </c>
-      <c r="B18">
+      <c r="C19">
         <v>1155.7</v>
       </c>
-      <c r="C18">
+      <c r="D19">
         <v>1159.3</v>
       </c>
-      <c r="D18">
+      <c r="E19">
         <v>1161.9000000000001</v>
       </c>
-      <c r="E18">
+      <c r="F19">
         <v>1166</v>
       </c>
-      <c r="F18">
+      <c r="G19">
         <v>1171.5999999999999</v>
       </c>
-      <c r="G18">
+      <c r="H19">
         <v>1177.4000000000001</v>
       </c>
-      <c r="H18">
+      <c r="I19">
         <v>1183.0999999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B20">
         <v>338</v>
       </c>
-      <c r="B19">
+      <c r="C20">
         <v>1155.9000000000001</v>
       </c>
-      <c r="C19">
+      <c r="D20">
         <v>1159.4000000000001</v>
       </c>
-      <c r="D19">
+      <c r="E20">
         <v>1162.0999999999999</v>
       </c>
-      <c r="E19">
-        <v>166.3</v>
-      </c>
-      <c r="F19">
+      <c r="F20">
+        <v>1166.3</v>
+      </c>
+      <c r="G20">
         <v>1171.9000000000001</v>
       </c>
-      <c r="G19">
+      <c r="H20">
         <v>1177.7</v>
       </c>
-      <c r="H19">
+      <c r="I20">
         <v>1183.3</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B21">
         <v>342</v>
       </c>
-      <c r="B20">
+      <c r="C21">
         <v>1156.0999999999999</v>
       </c>
-      <c r="C20">
+      <c r="D21">
         <v>1159.5999999999999</v>
       </c>
-      <c r="D20">
+      <c r="E21">
         <v>1162.3</v>
       </c>
-      <c r="E20">
+      <c r="F21">
         <v>1166.5</v>
       </c>
-      <c r="F20">
+      <c r="G21">
         <v>1172.0999999999999</v>
       </c>
-      <c r="G20">
+      <c r="H21">
         <v>1177.9000000000001</v>
       </c>
-      <c r="H20">
+      <c r="I21">
         <v>1183.5</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B22">
         <v>346</v>
       </c>
-      <c r="B21">
+      <c r="C22">
         <v>1156.3</v>
       </c>
-      <c r="C21">
+      <c r="D22">
         <v>1159.8</v>
       </c>
-      <c r="D21">
+      <c r="E22">
         <v>1162.5</v>
       </c>
-      <c r="E21">
+      <c r="F22">
         <v>1166.7</v>
       </c>
-      <c r="F21">
+      <c r="G22">
         <v>1172.3</v>
       </c>
-      <c r="G21">
+      <c r="H22">
         <v>1178.0999999999999</v>
       </c>
-      <c r="H21">
+      <c r="I22">
         <v>1183.8</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B23">
         <v>350</v>
       </c>
-      <c r="B22">
+      <c r="C23">
         <v>1156.5</v>
       </c>
-      <c r="C22">
+      <c r="D23">
         <v>1160</v>
       </c>
-      <c r="D22">
+      <c r="E23">
         <v>1162.5999999999999</v>
       </c>
-      <c r="E22">
+      <c r="F23">
         <v>1166.9000000000001</v>
       </c>
-      <c r="F22">
+      <c r="G23">
         <v>1172.5</v>
       </c>
-      <c r="G22">
+      <c r="H23">
         <v>1178.3</v>
       </c>
-      <c r="H22">
+      <c r="I23">
         <v>1184</v>
       </c>
     </row>

</xml_diff>